<commit_message>
Actualizacion de formatos y mejoras en para la generacion de SCPM-07 y exportacion de plantilla para STPS basandose en si el trabajador estado dado de baja
</commit_message>
<xml_diff>
--- a/backend/outputs/50693527/50693527_EVENTO_SCPM-07.xlsx
+++ b/backend/outputs/50693527/50693527_EVENTO_SCPM-07.xlsx
@@ -2739,27 +2739,15 @@
       <c r="H30" s="171" t="n"/>
       <c r="I30" s="27" t="inlineStr">
         <is>
-          <t>375714</t>
-        </is>
-      </c>
-      <c r="J30" s="27" t="inlineStr">
-        <is>
-          <t>580429</t>
-        </is>
-      </c>
-      <c r="K30" s="27" t="inlineStr">
-        <is>
-          <t>377388</t>
-        </is>
-      </c>
-      <c r="L30" s="27" t="inlineStr">
-        <is>
-          <t>549311</t>
-        </is>
-      </c>
+          <t>{% tr %}{% for participante in lista_participantes %}{{ participante.ficha }}</t>
+        </is>
+      </c>
+      <c r="J30" s="27" t="n"/>
+      <c r="K30" s="27" t="n"/>
+      <c r="L30" s="27" t="n"/>
       <c r="M30" s="27" t="inlineStr">
         <is>
-          <t>372629</t>
+          <t>{% endfor %}</t>
         </is>
       </c>
       <c r="N30" s="131" t="n"/>
@@ -2775,29 +2763,13 @@
       <c r="H31" s="174" t="n"/>
       <c r="I31" s="28" t="inlineStr">
         <is>
-          <t>Almazan Sanchez Adolfo Rene</t>
-        </is>
-      </c>
-      <c r="J31" s="28" t="inlineStr">
-        <is>
-          <t>Almazan Sanchez Arturo Raul</t>
-        </is>
-      </c>
-      <c r="K31" s="28" t="inlineStr">
-        <is>
-          <t>Barajas Rocha Mayra Jhoana</t>
-        </is>
-      </c>
-      <c r="L31" s="28" t="inlineStr">
-        <is>
-          <t>Bravo Velez Yadira</t>
-        </is>
-      </c>
-      <c r="M31" s="28" t="inlineStr">
-        <is>
-          <t>Garcia Galvan Mariel</t>
-        </is>
-      </c>
+          <t>{{ paticipante.nombe_completo }}</t>
+        </is>
+      </c>
+      <c r="J31" s="28" t="n"/>
+      <c r="K31" s="28" t="n"/>
+      <c r="L31" s="28" t="n"/>
+      <c r="M31" s="28" t="n"/>
       <c r="N31" s="131" t="n"/>
     </row>
     <row r="32" ht="16.5" customHeight="1">

</xml_diff>